<commit_message>
Expand FMCG/F&B HCMC sourcing: 18 job-seeking candidates
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JmMXk4GVdXerQikF6zQVcP
</commit_message>
<xml_diff>
--- a/sourcing/2026-10-08-truong-phong-kinh-doanh-fmcg-fnb-hcm/ung-vien-truong-phong-kinh-doanh-fmcg-fnb-hcm.xlsx
+++ b/sourcing/2026-10-08-truong-phong-kinh-doanh-fmcg-fnb-hcm/ung-vien-truong-phong-kinh-doanh-fmcg-fnb-hcm.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Hướng dẫn" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ứng viên'!$A$1:$U$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ứng viên'!$A$1:$U$27</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U12"/>
+  <dimension ref="A1:U27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -640,32 +640,32 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>FMCG-001</t>
+          <t>FMCG-008</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Ben Nguyen</t>
+          <t>Nguyen Minh Hoang</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>HORECA Sales Manager (01/2021–06/2023)</t>
+          <t>Commercial &amp; Sales Director; Board Member</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Saigon Baigur (beer)</t>
+          <t>Hochiminh Food &amp; Beverage Associates</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Not verified (worked at a Saigon brand)</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>F&amp;B/beverage, HORECA channel; leader experience in sales and distributor coaching</t>
+          <t>F&amp;B, commercial/sales director level</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -680,25 +680,25 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Profile headline: "Looking for a new job"</t>
+          <t>Profile: "Currently looking for a senior operating role (CEO / CMO / Commercial Director / Sales Director)..."</t>
         </is>
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>https://vn.linkedin.com/in/ben-nguyen-2585b393</t>
+          <t>https://vn.linkedin.com/in/nguyen-minh-hoang-a776a9334</t>
         </is>
       </c>
       <c r="M2" s="2" t="n">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Current location not verified as HCM; Headline date unknown; Team size not stated</t>
+          <t>Senior level: may expect above a Department Head salary</t>
         </is>
       </c>
       <c r="O2" s="3" t="inlineStr">
         <is>
-          <t>https://vn.linkedin.com/in/ben-nguyen-2585b393</t>
+          <t>https://vn.linkedin.com/in/nguyen-minh-hoang-a776a9334</t>
         </is>
       </c>
       <c r="P2" s="4" t="inlineStr">
@@ -731,32 +731,32 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>FMCG-002</t>
+          <t>FMCG-011</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Khiem Quach</t>
+          <t>Justin Nguyen</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Sales Manager (since 2017), seeking Head Sales Manager</t>
+          <t>Sales Manager – Southern Region (since 03/2021)</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>International Cosmetic Company (ICC); previously International Dairy</t>
+          <t>PRAN-RFL Group (food &amp; beverage)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Not verified</t>
+          <t>Southern Region (likely HCM)</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>FMCG (cosmetics, dairy), Sales Manager for 9+ years</t>
+          <t>15+ years in sales and market development, recruiting and coaching the team, managing promotion programs</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -771,25 +771,25 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Profile headline: "Looking for Head Sales Manager"</t>
+          <t>Profile headline: "Looking for new opportunity"</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>https://vn.linkedin.com/in/khiem-quach-55a42927</t>
+          <t>https://vn.linkedin.com/in/justin-nguyen-03421092</t>
         </is>
       </c>
       <c r="M3" s="2" t="n">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Location not verified; Headline date unknown</t>
+          <t>Exact location (HCM) not confirmed</t>
         </is>
       </c>
       <c r="O3" s="3" t="inlineStr">
         <is>
-          <t>https://vn.linkedin.com/in/khiem-quach-55a42927</t>
+          <t>https://vn.linkedin.com/in/justin-nguyen-03421092</t>
         </is>
       </c>
       <c r="P3" s="4" t="inlineStr">
@@ -822,32 +822,32 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>FMCG-003</t>
+          <t>FMCG-010</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Thuan Hoa Nguyen</t>
+          <t>nhat nguyen the duc</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Freelance Trainer / E-commerce Advisor; previously Senior Key Account Manager, Lazada (2019–2023)</t>
+          <t>Head of Sales (since 09/2023); CCO at Delice Food; previously Sales Director</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Into The Tech (ITT)</t>
+          <t>FMCG Company / Delice Food</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Not verified</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>10+ years B2B/B2B2C, loyalty and e-commerce, worked with FMCG clients; not a direct FMCG sales manager</t>
+          <t>FMCG/food, Head of Sales, CCO, Sales Director</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -862,25 +862,25 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Profile headline: "Open to full-time leadership roles..."</t>
+          <t>Profile headline: "Open to work"</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>https://vn.linkedin.com/in/thuanhoanguyen</t>
+          <t>https://vn.linkedin.com/in/nhat-nguyen-the-duc-47664986</t>
         </is>
       </c>
       <c r="M4" s="2" t="n">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>Mainly e-commerce/KAM, not traditional FMCG GT/MT sales management</t>
+          <t>Location not verified; Senior level</t>
         </is>
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>https://vn.linkedin.com/in/thuanhoanguyen</t>
+          <t>https://vn.linkedin.com/in/nhat-nguyen-the-duc-47664986</t>
         </is>
       </c>
       <c r="P4" s="4" t="inlineStr">
@@ -913,32 +913,32 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>FMCG-004</t>
+          <t>FMCG-002</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Thanh Do Trung</t>
+          <t>Khiem Quach</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Sales &amp; distribution (10+ years)</t>
+          <t>Sales Manager (since 2017), seeking Head Sales Manager</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>(not stated)</t>
+          <t>International Cosmetic Company (ICC); previously International Dairy</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Not verified</t>
+          <t>Likely HCM (Regional Sales Manager at Nestlé, HCM East, 2014–2016)</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>FMCG, beer/beverage, coffee, household appliances</t>
+          <t>FMCG (cosmetics, dairy), Sales Manager for 9+ years; previously RSM at Nestlé HCM (East)</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -953,25 +953,25 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Profile headline: "Looking for a new job opportunity."</t>
+          <t>Profile headline: "Looking for Head Sales Manager"</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>https://vn.linkedin.com/in/thanh-do-trung-15714335</t>
+          <t>https://vn.linkedin.com/in/khiem-quach-55a42927</t>
         </is>
       </c>
       <c r="M5" s="2" t="n">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Management level and location not verified; Headline date unknown</t>
+          <t>Current location not confirmed (previously worked in HCM); Headline date unknown</t>
         </is>
       </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
-          <t>https://vn.linkedin.com/in/thanh-do-trung-15714335</t>
+          <t>https://vn.linkedin.com/in/khiem-quach-55a42927</t>
         </is>
       </c>
       <c r="P5" s="4" t="inlineStr">
@@ -1004,32 +1004,32 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>FMCG-005</t>
+          <t>FMCG-009</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Dat Tran</t>
+          <t>Nguyễn Phi Vũ</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Seeking a Sales Manager role</t>
+          <t>On Premise Senior Executive</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>(pharmaceuticals)</t>
+          <t>Suntory PepsiCo Vietnam Beverage</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Not verified</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>15 years of management in pharmaceuticals (ETC &amp; OTC), built sales teams; OTC is close to FMCG</t>
+          <t>8+ years in sales, FMCG beverages, Horeca/On-premise channel</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -1044,25 +1044,25 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Profile headline: "Looking for new role as a Sales Manager"</t>
+          <t>Profile headline: "Looking for sales manager position (B2B/ Horeca/ FMCG/ or High Technology products for Horeca)"</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>https://vn.linkedin.com/in/dat-tran-30b444136</t>
+          <t>https://vn.linkedin.com/in/nguy%E1%BB%85n-phi-v%C5%A9</t>
         </is>
       </c>
       <c r="M6" s="2" t="n">
-        <v>50</v>
+        <v>72</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>Pharmaceuticals, not FMCG/F&amp;B; Location not verified</t>
+          <t>Currently Senior Executive: first step up to Manager; Team management not verified</t>
         </is>
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>https://vn.linkedin.com/in/dat-tran-30b444136</t>
+          <t>https://vn.linkedin.com/in/nguy%E1%BB%85n-phi-v%C5%A9</t>
         </is>
       </c>
       <c r="P6" s="4" t="inlineStr">
@@ -1095,22 +1095,22 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>FMCG-006</t>
+          <t>FMCG-012</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Việt Tiến</t>
+          <t>Nhan Vo</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Sales Supervisor, seeking ASM</t>
+          <t>Seeking a Sales Director role</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>(FMCG)</t>
+          <t>Suntory PepsiCo Vietnam Beverage</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>7 years FMCG, supervisor level</t>
+          <t>FMCG beverages (Suntory PepsiCo)</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -1135,25 +1135,25 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Profile headline: "Sales Supervisor | 7 Years FMCG | Seeking ASM Opportunity"</t>
+          <t>Profile headline: "Looking for Sales Director position"</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>https://vn.linkedin.com/in/vi%E1%BB%87t-ti%E1%BA%BFn-4b62a23b8</t>
+          <t>https://vn.linkedin.com/in/nhan-vo-86087ab1</t>
         </is>
       </c>
       <c r="M7" s="2" t="n">
-        <v>45</v>
+        <v>68</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>Supervisor level, below Department Head; Location not verified</t>
+          <t>Current title and location not verified</t>
         </is>
       </c>
       <c r="O7" s="3" t="inlineStr">
         <is>
-          <t>https://vn.linkedin.com/in/vi%E1%BB%87t-ti%E1%BA%BFn-4b62a23b8</t>
+          <t>https://vn.linkedin.com/in/nhan-vo-86087ab1</t>
         </is>
       </c>
       <c r="P7" s="4" t="inlineStr">
@@ -1186,32 +1186,32 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>FMCG-007</t>
+          <t>FMCG-001</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Thuỳ Dung</t>
+          <t>Ben Nguyen</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Seeking Area Sales Manager</t>
+          <t>HORECA Sales Manager (01/2021–06/2023)</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>(FMCG)</t>
+          <t>Saigon Baigur (beer)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Not verified</t>
+          <t>Not verified (worked at a Saigon brand)</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>FMCG; previously reported to an ASM (sub-ASM level)</t>
+          <t>F&amp;B/beverage, HORECA channel; leader experience in sales and distributor coaching</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -1226,25 +1226,25 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Profile headline: "Looking for Area Sales Manager"</t>
+          <t>Profile headline: "Looking for a new job"</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>https://vn.linkedin.com/in/thu%E1%BB%B3-dung-26877b16a</t>
+          <t>https://vn.linkedin.com/in/ben-nguyen-2585b393</t>
         </is>
       </c>
       <c r="M8" s="2" t="n">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>Level below ASM; Location not verified</t>
+          <t>Current location not verified as HCM; Headline date unknown; Team size not stated</t>
         </is>
       </c>
       <c r="O8" s="3" t="inlineStr">
         <is>
-          <t>https://vn.linkedin.com/in/thu%E1%BB%B3-dung-26877b16a</t>
+          <t>https://vn.linkedin.com/in/ben-nguyen-2585b393</t>
         </is>
       </c>
       <c r="P8" s="4" t="inlineStr">
@@ -1272,60 +1272,70 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Theo dõi</t>
+          <t>Chính</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>FMCG-W01</t>
+          <t>FMCG-017</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>HOP DANG</t>
+          <t>Phan Xuan Thuong</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Area Sales Manager (since 12/2024)</t>
+          <t>Regional Sales Manager | MBA</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>LOF International Dairy JSC</t>
+          <t>Reckitt</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Ho Chi Minh City Metropolitan Area</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>ASM in the dairy industry, HCM</t>
+          <t>FMCG (Reckitt), RSM</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>unverified</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr"/>
+          <t>probable</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>không rõ</t>
+        </is>
+      </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Chưa thấy tín hiệu tìm việc công khai</t>
-        </is>
-      </c>
-      <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="2" t="n"/>
+          <t>Profile summary: "I am looking for a challenging job in Sales..." (may be an old summary)</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/phanxuanthuong</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="n">
+        <v>65</v>
+      </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>Cần hỏi trực tiếp nhu cầu chuyển việc</t>
+          <t>Signal may be an old summary line, need to confirm</t>
         </is>
       </c>
       <c r="O9" s="3" t="inlineStr">
         <is>
-          <t>https://vn.linkedin.com/in/hop-dang-68bb35312</t>
+          <t>https://vn.linkedin.com/in/phanxuanthuong</t>
         </is>
       </c>
       <c r="P9" s="4" t="inlineStr">
@@ -1353,27 +1363,27 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Theo dõi</t>
+          <t>Chính</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>FMCG-W02</t>
+          <t>FMCG-013</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Hoa Nguyen</t>
+          <t>Thái Tường Trần</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Area Sales Manager</t>
+          <t>Previously Regional Sales Manager, Retail Account Manager</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Tribeco Vietnam (beverages)</t>
+          <t>(supplementary food, ICT...)</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1383,30 +1393,40 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>FMCG sales, 13 years in management, 4+ years as ASM</t>
+          <t>RSM, retail account, new channel development for supplementary food</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>unverified</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr"/>
+          <t>confirmed</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>không rõ</t>
+        </is>
+      </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Chưa thấy tín hiệu tìm việc công khai</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr"/>
-      <c r="M10" s="2" t="n"/>
+          <t>Profile headline: "looking for new opportunity in Sales Manager, RSM"</t>
+        </is>
+      </c>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/th%C3%A1i-t%C6%B0%E1%BB%9Dng-tr%E1%BA%A7n-3aa884427</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="n">
+        <v>62</v>
+      </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>Cần hỏi trực tiếp nhu cầu chuyển việc</t>
+          <t>Location not verified; Mixed industry experience (supplementary food, ICT)</t>
         </is>
       </c>
       <c r="O10" s="3" t="inlineStr">
         <is>
-          <t>https://vn.linkedin.com/in/hoa-nguyen-881045132</t>
+          <t>https://vn.linkedin.com/in/th%C3%A1i-t%C6%B0%E1%BB%9Dng-tr%E1%BA%A7n-3aa884427</t>
         </is>
       </c>
       <c r="P10" s="4" t="inlineStr">
@@ -1434,60 +1454,70 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Theo dõi</t>
+          <t>Chính</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>FMCG-W03</t>
+          <t>FMCG-014</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Phung Ngoc Trang</t>
+          <t>Dinh Thanh Hai</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Vice President; previously National Sales Manager at Richfield Worldwide (2023–2024)</t>
+          <t>ASM</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Hung Viet Fishsauce</t>
+          <t>Nestlé</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Not verified</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>27 years of experience, Head of Sales &amp; Sales Coach; senior level</t>
+          <t>10+ years FMCG, ASM at Nestlé</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>unverified</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr"/>
+          <t>probable</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>không rõ</t>
+        </is>
+      </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Chưa thấy tín hiệu tìm việc công khai</t>
-        </is>
-      </c>
-      <c r="L11" s="2" t="inlineStr"/>
-      <c r="M11" s="2" t="n"/>
+          <t>Profile summary: "...10 years of experience in FMCG... willing to join a new environment"</t>
+        </is>
+      </c>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/dinh-thanh-hai-820093188</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="n">
+        <v>62</v>
+      </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>Cần hỏi trực tiếp nhu cầu chuyển việc</t>
+          <t>Not an explicit Open to Work; Location not verified</t>
         </is>
       </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
-          <t>https://vn.linkedin.com/in/phung-ngoc-trang-3651116</t>
+          <t>https://vn.linkedin.com/in/dinh-thanh-hai-820093188</t>
         </is>
       </c>
       <c r="P11" s="4" t="inlineStr">
@@ -1515,60 +1545,70 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Theo dõi</t>
+          <t>Chính</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>FMCG-W04</t>
+          <t>FMCG-015</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Ms. Many</t>
+          <t>Trinh Nguyen (Tawan)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Sales Manager</t>
+          <t>Senior Key Account Manager</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Huynh Lam Natural Products Manufacturing</t>
+          <t>SABECO</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City Metropolitan Area</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Supplies natural ingredients to F&amp;B chains worldwide; display name is not a full name</t>
+          <t>Beer/beverage FMCG, Modern Trade key accounts</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>unverified</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr"/>
+          <t>probable</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>không rõ</t>
+        </is>
+      </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Chưa thấy tín hiệu tìm việc công khai</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr"/>
-      <c r="M12" s="2" t="n"/>
+          <t>Profile headline lists target roles: "...Sales Manager | Commercial Manager | Modern Trade Manager | Regional/International Key Account roles"</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/nguyen-chau-mong-trinh</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>62</v>
+      </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>Cần hỏi trực tiếp nhu cầu chuyển việc</t>
+          <t>Headline lists target roles but the snippet is cut off, need to confirm OTW</t>
         </is>
       </c>
       <c r="O12" s="3" t="inlineStr">
         <is>
-          <t>https://vn.linkedin.com/in/ms-many-b61937376</t>
+          <t>https://vn.linkedin.com/in/nguyen-chau-mong-trinh</t>
         </is>
       </c>
       <c r="P12" s="4" t="inlineStr">
@@ -1590,32 +1630,1317 @@
       </c>
       <c r="U12" s="4" t="n"/>
     </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Chính</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>FMCG-003</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Thuan Hoa Nguyen</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Freelance Trainer / E-commerce Advisor; previously Senior Key Account Manager, Lazada (2019–2023)</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Into The Tech (ITT)</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>10+ years B2B/B2B2C, loyalty and e-commerce, worked with FMCG clients; not a direct FMCG sales manager</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>confirmed</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>không rõ</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Profile headline: "Open to full-time leadership roles..."</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/thuanhoanguyen</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>Mainly e-commerce/KAM, not traditional FMCG GT/MT sales management</t>
+        </is>
+      </c>
+      <c r="O13" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/thuanhoanguyen</t>
+        </is>
+      </c>
+      <c r="P13" s="4" t="inlineStr">
+        <is>
+          <t>Chưa liên hệ</t>
+        </is>
+      </c>
+      <c r="Q13" s="5" t="n"/>
+      <c r="R13" s="4" t="n"/>
+      <c r="S13" s="4" t="inlineStr">
+        <is>
+          <t>Chưa phản hồi</t>
+        </is>
+      </c>
+      <c r="T13" s="4" t="inlineStr">
+        <is>
+          <t>Chưa xác minh</t>
+        </is>
+      </c>
+      <c r="U13" s="4" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Chính</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>FMCG-018</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Ngo Manh Hung</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Go to Market Specialist FMCG; previously Southern Sales Manager (automotive)</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>(tobacco, 19 years)</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Not verified</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>19 years in tobacco (FMCG) + 3 years Southern Sales Manager</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>probable</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>không rõ</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Profile shows "Available for new opportunity" (in the experience section)</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/ngo-manh-hung-850a2461</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>Unclear wording, date unknown; Location not verified</t>
+        </is>
+      </c>
+      <c r="O14" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/ngo-manh-hung-850a2461</t>
+        </is>
+      </c>
+      <c r="P14" s="4" t="inlineStr">
+        <is>
+          <t>Chưa liên hệ</t>
+        </is>
+      </c>
+      <c r="Q14" s="5" t="n"/>
+      <c r="R14" s="4" t="n"/>
+      <c r="S14" s="4" t="inlineStr">
+        <is>
+          <t>Chưa phản hồi</t>
+        </is>
+      </c>
+      <c r="T14" s="4" t="inlineStr">
+        <is>
+          <t>Chưa xác minh</t>
+        </is>
+      </c>
+      <c r="U14" s="4" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Chính</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>FMCG-016</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>DUNG NGUYEN THI MY</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Key Account Manager</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>(FMCG – Modern Trade)</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Not verified</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>KAM FMCG, Modern Trade channel, led strategic accounts</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>probable</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>không rõ</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Profile summary: "...I'm looking for a company where I can further..."</t>
+        </is>
+      </c>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/dung-nguyen-thi-my-4a6493234</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>Signal is only a summary phrase; Location not verified</t>
+        </is>
+      </c>
+      <c r="O15" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/dung-nguyen-thi-my-4a6493234</t>
+        </is>
+      </c>
+      <c r="P15" s="4" t="inlineStr">
+        <is>
+          <t>Chưa liên hệ</t>
+        </is>
+      </c>
+      <c r="Q15" s="5" t="n"/>
+      <c r="R15" s="4" t="n"/>
+      <c r="S15" s="4" t="inlineStr">
+        <is>
+          <t>Chưa phản hồi</t>
+        </is>
+      </c>
+      <c r="T15" s="4" t="inlineStr">
+        <is>
+          <t>Chưa xác minh</t>
+        </is>
+      </c>
+      <c r="U15" s="4" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Chính</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>FMCG-005</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Dat Tran</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Seeking a Sales Manager role</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>(pharmaceuticals)</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Not verified</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>15 years of management in pharmaceuticals (ETC &amp; OTC), built sales teams; OTC is close to FMCG</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>confirmed</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>không rõ</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Profile headline: "Looking for new role as a Sales Manager"</t>
+        </is>
+      </c>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/dat-tran-30b444136</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>Pharmaceuticals, not FMCG/F&amp;B; Location not verified</t>
+        </is>
+      </c>
+      <c r="O16" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/dat-tran-30b444136</t>
+        </is>
+      </c>
+      <c r="P16" s="4" t="inlineStr">
+        <is>
+          <t>Chưa liên hệ</t>
+        </is>
+      </c>
+      <c r="Q16" s="5" t="n"/>
+      <c r="R16" s="4" t="n"/>
+      <c r="S16" s="4" t="inlineStr">
+        <is>
+          <t>Chưa phản hồi</t>
+        </is>
+      </c>
+      <c r="T16" s="4" t="inlineStr">
+        <is>
+          <t>Chưa xác minh</t>
+        </is>
+      </c>
+      <c r="U16" s="4" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Chính</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>FMCG-006</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Việt Tiến</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Sales Supervisor, seeking ASM</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>(FMCG)</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Not verified</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>7 years FMCG, supervisor level</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>confirmed</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>không rõ</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Profile headline: "Sales Supervisor | 7 Years FMCG | Seeking ASM Opportunity"</t>
+        </is>
+      </c>
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/vi%E1%BB%87t-ti%E1%BA%BFn-4b62a23b8</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>Supervisor level, below Department Head; Location not verified</t>
+        </is>
+      </c>
+      <c r="O17" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/vi%E1%BB%87t-ti%E1%BA%BFn-4b62a23b8</t>
+        </is>
+      </c>
+      <c r="P17" s="4" t="inlineStr">
+        <is>
+          <t>Chưa liên hệ</t>
+        </is>
+      </c>
+      <c r="Q17" s="5" t="n"/>
+      <c r="R17" s="4" t="n"/>
+      <c r="S17" s="4" t="inlineStr">
+        <is>
+          <t>Chưa phản hồi</t>
+        </is>
+      </c>
+      <c r="T17" s="4" t="inlineStr">
+        <is>
+          <t>Chưa xác minh</t>
+        </is>
+      </c>
+      <c r="U17" s="4" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Chính</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>FMCG-019</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Richard Pham</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Sales Specialist | Foodservice &amp; Bakery Solutions</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>(food ingredients)</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Not verified</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Foodservice/bakery, FMCG</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>confirmed</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>không rõ</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Profile: "Currently, I am looking for opportunities to grow into Area Sales Manager or Business Development Manager positions within FMCG, Food Ingredients, Dairy..."</t>
+        </is>
+      </c>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/richard-pham-187288188</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>Specialist level, below Department Head; Location not verified</t>
+        </is>
+      </c>
+      <c r="O18" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/richard-pham-187288188</t>
+        </is>
+      </c>
+      <c r="P18" s="4" t="inlineStr">
+        <is>
+          <t>Chưa liên hệ</t>
+        </is>
+      </c>
+      <c r="Q18" s="5" t="n"/>
+      <c r="R18" s="4" t="n"/>
+      <c r="S18" s="4" t="inlineStr">
+        <is>
+          <t>Chưa phản hồi</t>
+        </is>
+      </c>
+      <c r="T18" s="4" t="inlineStr">
+        <is>
+          <t>Chưa xác minh</t>
+        </is>
+      </c>
+      <c r="U18" s="4" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Chính</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>FMCG-007</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Thuỳ Dung</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Seeking Area Sales Manager</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>(FMCG)</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Not verified</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>FMCG; previously reported to an ASM (sub-ASM level)</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>confirmed</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>không rõ</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Profile headline: "Looking for Area Sales Manager"</t>
+        </is>
+      </c>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/thu%E1%BB%B3-dung-26877b16a</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>Level below ASM; Location not verified</t>
+        </is>
+      </c>
+      <c r="O19" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/thu%E1%BB%B3-dung-26877b16a</t>
+        </is>
+      </c>
+      <c r="P19" s="4" t="inlineStr">
+        <is>
+          <t>Chưa liên hệ</t>
+        </is>
+      </c>
+      <c r="Q19" s="5" t="n"/>
+      <c r="R19" s="4" t="n"/>
+      <c r="S19" s="4" t="inlineStr">
+        <is>
+          <t>Chưa phản hồi</t>
+        </is>
+      </c>
+      <c r="T19" s="4" t="inlineStr">
+        <is>
+          <t>Chưa xác minh</t>
+        </is>
+      </c>
+      <c r="U19" s="4" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Theo dõi</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>FMCG-W01</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>HOP DANG</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Area Sales Manager (since 12/2024)</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>LOF International Dairy JSC</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>ASM in the dairy industry, HCM</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Chưa thấy tín hiệu tìm việc công khai</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="n"/>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>Cần hỏi trực tiếp nhu cầu chuyển việc</t>
+        </is>
+      </c>
+      <c r="O20" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/hop-dang-68bb35312</t>
+        </is>
+      </c>
+      <c r="P20" s="4" t="inlineStr">
+        <is>
+          <t>Chưa liên hệ</t>
+        </is>
+      </c>
+      <c r="Q20" s="5" t="n"/>
+      <c r="R20" s="4" t="n"/>
+      <c r="S20" s="4" t="inlineStr">
+        <is>
+          <t>Chưa phản hồi</t>
+        </is>
+      </c>
+      <c r="T20" s="4" t="inlineStr">
+        <is>
+          <t>Chưa xác minh</t>
+        </is>
+      </c>
+      <c r="U20" s="4" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Theo dõi</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>FMCG-W02</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Hoa Nguyen</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Area Sales Manager</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Tribeco Vietnam (beverages)</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Not verified</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>FMCG sales, 13 years in management, 4+ years as ASM</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Chưa thấy tín hiệu tìm việc công khai</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="n"/>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>Cần hỏi trực tiếp nhu cầu chuyển việc</t>
+        </is>
+      </c>
+      <c r="O21" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/hoa-nguyen-881045132</t>
+        </is>
+      </c>
+      <c r="P21" s="4" t="inlineStr">
+        <is>
+          <t>Chưa liên hệ</t>
+        </is>
+      </c>
+      <c r="Q21" s="5" t="n"/>
+      <c r="R21" s="4" t="n"/>
+      <c r="S21" s="4" t="inlineStr">
+        <is>
+          <t>Chưa phản hồi</t>
+        </is>
+      </c>
+      <c r="T21" s="4" t="inlineStr">
+        <is>
+          <t>Chưa xác minh</t>
+        </is>
+      </c>
+      <c r="U21" s="4" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Theo dõi</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>FMCG-W03</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Phung Ngoc Trang</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Vice President; previously National Sales Manager at Richfield Worldwide (2023–2024)</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Hung Viet Fishsauce</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>27 years of experience, Head of Sales &amp; Sales Coach; senior level</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Chưa thấy tín hiệu tìm việc công khai</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr"/>
+      <c r="M22" s="2" t="n"/>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>Cần hỏi trực tiếp nhu cầu chuyển việc</t>
+        </is>
+      </c>
+      <c r="O22" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/phung-ngoc-trang-3651116</t>
+        </is>
+      </c>
+      <c r="P22" s="4" t="inlineStr">
+        <is>
+          <t>Chưa liên hệ</t>
+        </is>
+      </c>
+      <c r="Q22" s="5" t="n"/>
+      <c r="R22" s="4" t="n"/>
+      <c r="S22" s="4" t="inlineStr">
+        <is>
+          <t>Chưa phản hồi</t>
+        </is>
+      </c>
+      <c r="T22" s="4" t="inlineStr">
+        <is>
+          <t>Chưa xác minh</t>
+        </is>
+      </c>
+      <c r="U22" s="4" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Theo dõi</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>FMCG-W04</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Ms. Many</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Sales Manager</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Huynh Lam Natural Products Manufacturing</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City Metropolitan Area</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Supplies natural ingredients to F&amp;B chains worldwide; display name is not a full name</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Chưa thấy tín hiệu tìm việc công khai</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="n"/>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>Cần hỏi trực tiếp nhu cầu chuyển việc</t>
+        </is>
+      </c>
+      <c r="O23" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/ms-many-b61937376</t>
+        </is>
+      </c>
+      <c r="P23" s="4" t="inlineStr">
+        <is>
+          <t>Chưa liên hệ</t>
+        </is>
+      </c>
+      <c r="Q23" s="5" t="n"/>
+      <c r="R23" s="4" t="n"/>
+      <c r="S23" s="4" t="inlineStr">
+        <is>
+          <t>Chưa phản hồi</t>
+        </is>
+      </c>
+      <c r="T23" s="4" t="inlineStr">
+        <is>
+          <t>Chưa xác minh</t>
+        </is>
+      </c>
+      <c r="U23" s="4" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Theo dõi</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>FMCG-W05</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Thinh Le</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Commercial Development Director; Sales Director FMCG</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>SIBC (Ex-PepsiCo, Ex-Masan)</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City Metropolitan Area</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>20+ years FMCG, strong in GT expansion and turnarounds</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Chưa thấy tín hiệu tìm việc công khai</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="n"/>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>Cần hỏi trực tiếp nhu cầu chuyển việc</t>
+        </is>
+      </c>
+      <c r="O24" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/thinh-le-3b679070</t>
+        </is>
+      </c>
+      <c r="P24" s="4" t="inlineStr">
+        <is>
+          <t>Chưa liên hệ</t>
+        </is>
+      </c>
+      <c r="Q24" s="5" t="n"/>
+      <c r="R24" s="4" t="n"/>
+      <c r="S24" s="4" t="inlineStr">
+        <is>
+          <t>Chưa phản hồi</t>
+        </is>
+      </c>
+      <c r="T24" s="4" t="inlineStr">
+        <is>
+          <t>Chưa xác minh</t>
+        </is>
+      </c>
+      <c r="U24" s="4" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Theo dõi</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>FMCG-W06</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Chung Nguyen</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Sales Director</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>FrieslandCampina (previously Mondelez)</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City Metropolitan Area</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Summary mentions 'looking for new opportunities to learn, grow...' (generic, not OTW)</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Chưa thấy tín hiệu tìm việc công khai</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr"/>
+      <c r="M25" s="2" t="n"/>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>Cần hỏi trực tiếp nhu cầu chuyển việc</t>
+        </is>
+      </c>
+      <c r="O25" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/chung-nguyen-9924681b</t>
+        </is>
+      </c>
+      <c r="P25" s="4" t="inlineStr">
+        <is>
+          <t>Chưa liên hệ</t>
+        </is>
+      </c>
+      <c r="Q25" s="5" t="n"/>
+      <c r="R25" s="4" t="n"/>
+      <c r="S25" s="4" t="inlineStr">
+        <is>
+          <t>Chưa phản hồi</t>
+        </is>
+      </c>
+      <c r="T25" s="4" t="inlineStr">
+        <is>
+          <t>Chưa xác minh</t>
+        </is>
+      </c>
+      <c r="U25" s="4" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Theo dõi</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>FMCG-W07</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Uyen Nguyen</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Horeca Sales Manager</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Annam Group</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Foodservice key accounts</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Chưa thấy tín hiệu tìm việc công khai</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="n"/>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>Cần hỏi trực tiếp nhu cầu chuyển việc</t>
+        </is>
+      </c>
+      <c r="O26" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/uyen-nguyen-b9a5801aa</t>
+        </is>
+      </c>
+      <c r="P26" s="4" t="inlineStr">
+        <is>
+          <t>Chưa liên hệ</t>
+        </is>
+      </c>
+      <c r="Q26" s="5" t="n"/>
+      <c r="R26" s="4" t="n"/>
+      <c r="S26" s="4" t="inlineStr">
+        <is>
+          <t>Chưa phản hồi</t>
+        </is>
+      </c>
+      <c r="T26" s="4" t="inlineStr">
+        <is>
+          <t>Chưa xác minh</t>
+        </is>
+      </c>
+      <c r="U26" s="4" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Theo dõi</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>FMCG-W08</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Ai Vo Tran Dau</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Sales Manager Food APAC</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Crespel &amp; Deiters Food Solutions</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Food ingredients B2B</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Chưa thấy tín hiệu tìm việc công khai</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr"/>
+      <c r="M27" s="2" t="n"/>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>Cần hỏi trực tiếp nhu cầu chuyển việc</t>
+        </is>
+      </c>
+      <c r="O27" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/votrandauai</t>
+        </is>
+      </c>
+      <c r="P27" s="4" t="inlineStr">
+        <is>
+          <t>Chưa liên hệ</t>
+        </is>
+      </c>
+      <c r="Q27" s="5" t="n"/>
+      <c r="R27" s="4" t="n"/>
+      <c r="S27" s="4" t="inlineStr">
+        <is>
+          <t>Chưa phản hồi</t>
+        </is>
+      </c>
+      <c r="T27" s="4" t="inlineStr">
+        <is>
+          <t>Chưa xác minh</t>
+        </is>
+      </c>
+      <c r="U27" s="4" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U12"/>
-  <conditionalFormatting sqref="P2:P12">
+  <autoFilter ref="A1:U27"/>
+  <conditionalFormatting sqref="P2:P27">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Đã liên hệ"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T2:T12">
+  <conditionalFormatting sqref="T2:T27">
     <cfRule type="cellIs" priority="2" operator="equal" dxfId="0">
       <formula>"Đang tìm việc"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="5">
-    <dataValidation sqref="P2:P12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="P2:P27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Chưa liên hệ,Đã liên hệ,Không liên hệ được"</formula1>
     </dataValidation>
-    <dataValidation sqref="R2:R12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="R2:R27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"LinkedIn InMail,LinkedIn kết nối,Email,Điện thoại/Zalo,Giới thiệu,Khác"</formula1>
     </dataValidation>
-    <dataValidation sqref="S2:S12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="S2:S27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Chưa phản hồi,Quan tâm,Không quan tâm,Hẹn phỏng vấn,Từ chối"</formula1>
     </dataValidation>
-    <dataValidation sqref="T2:T12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="T2:T27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Chưa xác minh,Đang tìm việc,Đang làm việc - mở cơ hội,Đang làm việc - không đổi việc,Đã nhận offer nơi khác"</formula1>
     </dataValidation>
-    <dataValidation sqref="Q2:Q12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date" operator="greaterThan">
+    <dataValidation sqref="Q2:Q27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date" operator="greaterThan">
       <formula1>DATE(2020,1,1)</formula1>
     </dataValidation>
   </dataValidations>
@@ -1634,10 +2959,36 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId44"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1675,7 +3026,7 @@
         </is>
       </c>
       <c r="B2" s="6">
-        <f>COUNTA('Ứng viên'!D2:D12)</f>
+        <f>COUNTA('Ứng viên'!D2:D27)</f>
         <v/>
       </c>
     </row>
@@ -1686,7 +3037,7 @@
         </is>
       </c>
       <c r="B3" s="6">
-        <f>COUNTIF('Ứng viên'!B2:B12,"Chính")</f>
+        <f>COUNTIF('Ứng viên'!B2:B27,"Chính")</f>
         <v/>
       </c>
     </row>
@@ -1697,7 +3048,7 @@
         </is>
       </c>
       <c r="B4" s="6">
-        <f>COUNTIF('Ứng viên'!I2:I12,"confirmed")</f>
+        <f>COUNTIF('Ứng viên'!I2:I27,"confirmed")</f>
         <v/>
       </c>
     </row>
@@ -1708,7 +3059,7 @@
         </is>
       </c>
       <c r="B5" s="6">
-        <f>COUNTIF('Ứng viên'!I2:I12,"probable")</f>
+        <f>COUNTIF('Ứng viên'!I2:I27,"probable")</f>
         <v/>
       </c>
     </row>
@@ -1719,7 +3070,7 @@
         </is>
       </c>
       <c r="B6" s="6">
-        <f>COUNTIF('Ứng viên'!B2:B12,"Theo dõi")</f>
+        <f>COUNTIF('Ứng viên'!B2:B27,"Theo dõi")</f>
         <v/>
       </c>
     </row>
@@ -1730,7 +3081,7 @@
         </is>
       </c>
       <c r="B7" s="6">
-        <f>COUNTIF('Ứng viên'!P2:P12,"Đã liên hệ")</f>
+        <f>COUNTIF('Ứng viên'!P2:P27,"Đã liên hệ")</f>
         <v/>
       </c>
     </row>
@@ -1741,7 +3092,7 @@
         </is>
       </c>
       <c r="B8" s="6">
-        <f>COUNTIF('Ứng viên'!P2:P12,"Chưa liên hệ")</f>
+        <f>COUNTIF('Ứng viên'!P2:P27,"Chưa liên hệ")</f>
         <v/>
       </c>
     </row>
@@ -1763,7 +3114,7 @@
         </is>
       </c>
       <c r="B10" s="6">
-        <f>COUNTIF('Ứng viên'!S2:S12,"Quan tâm")</f>
+        <f>COUNTIF('Ứng viên'!S2:S27,"Quan tâm")</f>
         <v/>
       </c>
     </row>
@@ -1774,7 +3125,7 @@
         </is>
       </c>
       <c r="B11" s="6">
-        <f>COUNTIF('Ứng viên'!S2:S12,"Hẹn phỏng vấn")</f>
+        <f>COUNTIF('Ứng viên'!S2:S27,"Hẹn phỏng vấn")</f>
         <v/>
       </c>
     </row>
@@ -1785,7 +3136,7 @@
         </is>
       </c>
       <c r="B12" s="6">
-        <f>COUNTIF('Ứng viên'!T2:T12,"Đang tìm việc")</f>
+        <f>COUNTIF('Ứng viên'!T2:T27,"Đang tìm việc")</f>
         <v/>
       </c>
     </row>
@@ -1796,7 +3147,7 @@
         </is>
       </c>
       <c r="B13" s="6">
-        <f>COUNTIF('Ứng viên'!T2:T12,"Chưa xác minh")</f>
+        <f>COUNTIF('Ứng viên'!T2:T27,"Chưa xác minh")</f>
         <v/>
       </c>
     </row>
@@ -1811,7 +3162,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1986,6 +3337,91 @@
       <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Anonymous; 13+ years FMCG GT, OTW for RSM+ but Central region</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Thanh Do Trung</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/thanh-do-trung-15714335</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Looking for a new job but experience is at HEINEKEN Hanoi Brewery, likely Hanoi; add back if they want to work in HCM</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Minh Pham</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/minh-pham-b43a79115</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Looking for Country/GM/Sales Manager but in power tools (Milwaukee), not FMCG</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Vo Tan Thanh</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/vo-tan-thanh-9534a8104</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Open for a new Sales Manager job but in packaging, not FMCG/F&amp;B</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Kim Hoang Nguyen</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/kimhoang279</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Looking for a new opportunity, HCM, but in plastics</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Annam Group Career / Hang Thanh Pham / Kieu Nguyen</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/annam-group-career-b56983108</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Recruiter headlines 'Looking for Sales Manager', not candidates</t>
         </is>
       </c>
     </row>
@@ -2000,6 +3436,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId14"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>